<commit_message>
Implemeted PID Control Without ant Library
</commit_message>
<xml_diff>
--- a/Parts_List.xlsx
+++ b/Parts_List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4af5cc2e0ff57d50/Acadamics/UOM Engineering/Academics/Semester 3/EN2533 Robot Design and  Competition/EN2533-Pulztrones/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4af5cc2e0ff57d50/Acadamics/UOM_Engineering/Academics/Semester-3/EN2533-Robot_Design_and_Competition/EN2533-Pulztrones/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{EBF8FB8B-7DFF-4E5D-9521-C69942F58029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{283E5B67-1650-40C9-AC35-71F18183922B}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{EBF8FB8B-7DFF-4E5D-9521-C69942F58029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E825C3EC-E7B4-4133-9D5B-E8D976F08F89}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F18862F5-15BA-408B-AD7A-40AC9A391A47}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{F18862F5-15BA-408B-AD7A-40AC9A391A47}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>Component Name</t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>Arduino Mega</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Raspberry pi</t>
+  </si>
+  <si>
+    <t>Pankaja</t>
   </si>
 </sst>
 </file>
@@ -132,6 +144,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -484,21 +500,37 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>